<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-03 Les raisins du gâteau
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-03.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-03.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine puis balcon</t>
+          <t>cuisine puis balcon, vanille, gâteau sur grille, raisins</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut poser des raisins en rond sur le gâteau. Il propose. Sarah dit non, puis je regarde, puis plus tard. Un raisin roule. Au balcon, il propose l'arrosoir. Sarah pose un raisin. Le rond est fini.</t>
+          <t>Le four rend un nuage de vanille. Un petit gâteau repose sur la grille. Sur un fil, un éclat de grille brille. Amir veut un rond de raisins, maintenant, avec Sarah. Il tend trop vite : le raisin roule, l'éclat saute. Il refuse de foncer, propose, accepte je regarde. Merci vécu. Au balcon, le gâteau glisse. Il attend. Sarah pose un raisin, s'arrête. L'éclat de grille tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La vanille chaude sort du four, toute douce. Un petit gâteau refroidit sur la grille. La grille fait un tout petit tic. Il a des trous, tout légers. Un bol de raisins secs attend. Les raisins sont sombres et un peu collants. Une cuillère de bois repose à côté. Tu as senti la vanille, Amir ? Oui, maman. C'est sucré. Les raisins sont prêts. Le gâteau aussi. On décore un peu, d'accord ? D'accord. Un rond de raisins. En ce moment, Amir tient un raisin. Il est collant, entre deux doigts. Maman ouvre la porte. Sarah arrive. Elle a une barrette bleue. Tu viens ? Non. Amir regarde papa. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Amir pose un raisin. Un autre raisin roule sous le bol. Il est parti. Tu as vu le raisin, Amir ? Oui. Amir penche le bol. Le raisin revient, tout collant. Tu proposes encore, tout doux ? Tu as vu le gâteau, Sarah ? Je regarde. Regarder, c'est une réponse.</t>
+          <t>Le four rend un nuage de vanille. Le nuage s'étale sur la vitre. La vitre donne sur le balcon. L'air du balcon entre, plus frais. Tu as senti la vanille, Amir ? Oui, maman. C'est sucré. On reste un moment, ici. La table est tiède, un peu collante. Un petit gâteau repose sur la grille. La grille fait un tic, très fin. Sur un fil, un éclat de grille brille. Il est blanc, maman. Tu le vois sur le fil ? Oui, il brille. C'est la grille du gâteau. Je veux un rond, maintenant ! Tes mains, Amir. On les passe sous l'eau. L'eau est tiède. Comme le gâteau. Un rond de raisins. Tu le veux autour ? Oui, autour. Près de la vanille, il peut reposer. Oui, près de la grille. Un bol de raisins attend au milieu. Les raisins sont sombres, un peu collants. Les raisins sont prêts. Le gâteau aussi. On décore un peu ? D'accord. En ce moment, Amir tient un raisin. Il est collant, entre deux doigts. Maman ouvre la porte. Sarah arrive. Elle a une barrette bleue. Tu viens ? Le rond, maintenant ! Non. Amir tend le raisin trop vite. Le raisin glisse sous le bol. Il est parti. L'éclat de grille saute près du bol. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le rond avec Sarah ? Oui, papa. Tes doigts sont collants ? Oui, maman. Tu tiens ma manche ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers Sarah. Je veux qu'elle pose un raisin !</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La vanille chaude sort du four, toute douce. Un petit gâteau refroidit sur la grille. La grille fait un tout petit tic. Il a des trous, tout légers. Un bol de raisins secs attend. Les raisins sont sombres et un peu collants. Une cuillère de bois repose à côté. Tu as senti la vanille, Amir ? Oui, maman. C'est sucré. Les raisins sont prêts. Le gâteau aussi. On décore un peu, d'accord ? D'accord. Un rond de raisins. En ce moment, Amir tient un raisin. Il est collant, entre deux doigts. Maman ouvre la porte. Sarah arrive. Elle a une barrette bleue. Tu viens ? Non. Amir regarde papa. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Amir pose un raisin. Un autre raisin roule sous le bol. Il est parti. Tu as vu le raisin, Amir ? Oui. Amir penche le bol. Le raisin revient, tout collant. Tu proposes encore, tout doux ? Tu as vu le gâteau, Sarah ? Je regarde. Regarder, c'est une réponse.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le four rend un nuage de vanille. Le nuage s'étale sur la vitre. La vitre donne sur le balcon. L'air du balcon entre, plus frais. Tu as senti la vanille, Amir ? Oui, maman. C'est sucré. On reste un moment, ici. La table est tiède, un peu collante. Un petit gâteau repose sur la grille. La grille fait un tic, très fin. Sur un fil, un &lt;emphasis level="moderate"&gt;éclat de grille&lt;/emphasis&gt; brille. Il est blanc, maman. Tu le vois sur le fil ? Oui, il brille. C'est la grille du gâteau. Je veux un rond, maintenant ! Tes mains, Amir. On les passe sous l'eau. L'eau est tiède. Comme le gâteau. Un rond de raisins. Tu le veux autour ? Oui, autour. Près de la vanille, il peut reposer. Oui, près de la grille. Un bol de raisins attend au milieu. Les raisins sont sombres, un peu collants. Les raisins sont prêts. Le gâteau aussi. On décore un peu ? D'accord. En ce moment, Amir tient un raisin. Il est collant, entre deux doigts. Maman ouvre la porte. Sarah arrive. Elle a une barrette bleue. Tu viens ? Le rond, maintenant ! Non. Amir tend le raisin trop vite. Le raisin glisse sous le bol. Il est parti. L'éclat de grille saute près du bol. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le rond avec Sarah ? Oui, papa. Tes doigts sont collants ? Oui, maman. Tu tiens ma manche ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers Sarah. Je veux qu'elle pose un raisin !&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Côme est dans le salon. Les crayons sont sur la table. Maman ouvre la porte. Dounia arrive. Côme veut dessiner. Il va &lt;emphasis&gt;proposer&lt;/emphasis&gt; un jeu. Côme dit : tu viens ? Dounia dit : non. Côme regarde maman. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Côme dit : d'accord. Il dessine un bateau. Dounia s'assoit près du canapé. Elle regarde. Côme laisse Dounia à sa place. Plus tard, au jardin, Côme se souvient. Il propose encore, tout doux. Côme dit : tu veux le cerceau ? Dounia dit : je regarde. Maman sourit. Maman dit : regarder, c'est une réponse. On peut accepter plusieurs réponses. Côme fait tourner le cerceau. Dounia avance un peu. Elle ne touche pas. C'est bien. Côme dit : plus tard, tu viens ? Dounia dit : plus tard. Côme dit : d'accord. Il continue. Maman chante tout bas. Dounia hoche la tête. Elle vient un moment. Puis elle s'arrête. Côme accepte. Maman dit : tu as su proposer. Tu as su accepter. Plusieurs réponses sont possibles. [pause]</t>
+          <t>Le four rend un nuage de vanille. Le nuage s'étale sur la vitre. La vitre donne sur le balcon. L'air du balcon entre, plus frais. Tu as senti la vanille, Amir ? Oui, maman. C'est sucré. On reste un moment, ici. La table est tiède, un peu collante. Un petit gâteau repose sur la grille. La grille fait un tic, très fin. Sur un fil, un &lt;emphasis&gt;éclat de grille&lt;/emphasis&gt; brille. Il est blanc, maman. Tu le vois sur le fil ? Oui, il brille. C'est la grille du gâteau. Je veux un rond, maintenant ! Tes mains, Amir. On les passe sous l'eau. L'eau est tiède. Comme le gâteau. Un rond de raisins. Tu le veux autour ? Oui, autour. Près de la vanille, il peut reposer. Oui, près de la grille. Un bol de raisins attend au milieu. Les raisins sont sombres, un peu collants. Les raisins sont prêts. Le gâteau aussi. On décore un peu ? D'accord. En ce moment, Amir tient un raisin. Il est collant, entre deux doigts. Maman ouvre la porte. Sarah arrive. Elle a une barrette bleue. Tu viens ? Le rond, maintenant ! Non. Amir tend le raisin trop vite. Le raisin glisse sous le bol. Il est parti. L'éclat de grille saute près du bol. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le rond avec Sarah ? Oui, papa. Tes doigts sont collants ? Oui, maman. Tu tiens ma manche ? Oui. Amir veut recommencer tout de suite. Ses doigts foncent vers Sarah. Je veux qu'elle pose un raisin ! [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>éclat de grille</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,55 +1326,75 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_rond_avec_sarah_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La vanille chaude sort du four, toute douce.
-narrateur|Un petit gâteau refroidit sur la grille.
-narrateur|La grille fait un tout petit tic.
-narrateur|Il a des trous, tout légers.
-narrateur|Un bol de raisins secs attend.
-narrateur|Les raisins sont sombres et un peu collants.
-narrateur|Une cuillère de bois repose à côté.
+          <t>narrateur|Le four rend un nuage de vanille.
+narrateur|Le nuage s'étale sur la vitre.
+narrateur|La vitre donne sur le balcon.
+narrateur|L'air du balcon entre, plus frais.
 maman|Tu as senti la vanille, Amir ?
 enfant-m|Oui, maman.
 enfant-m|C'est sucré.
+papa|On reste un moment, ici.
+narrateur|La table est tiède, un peu collante.
+narrateur|Un petit gâteau repose sur la grille.
+narrateur|La grille fait un tic, très fin.
+narrateur|Sur un fil, un éclat de grille brille.
+enfant-m|Il est blanc, maman.
+maman|Tu le vois sur le fil ?
+enfant-m|Oui, il brille.
+papa|C'est la grille du gâteau.
+enfant-m|Je veux un rond, maintenant !
+maman|Tes mains, Amir.
+maman|On les passe sous l'eau.
+enfant-m|L'eau est tiède.
+papa|Comme le gâteau.
+enfant-m|Un rond de raisins.
+maman|Tu le veux autour ?
+enfant-m|Oui, autour.
+papa|Près de la vanille, il peut reposer.
+enfant-m|Oui, près de la grille.
+narrateur|Un bol de raisins attend au milieu.
+narrateur|Les raisins sont sombres, un peu collants.
 papa|Les raisins sont prêts.
 papa|Le gâteau aussi.
-maman|On décore un peu, d'accord ?
+maman|On décore un peu ?
 enfant-m|D'accord.
-enfant-m|Un rond de raisins.
 narrateur|En ce moment, Amir tient un raisin.
 narrateur|Il est collant, entre deux doigts.
 narrateur|Maman ouvre la porte.
 narrateur|Sarah arrive.
 narrateur|Elle a une barrette bleue.
 enfant-m|Tu viens ?
+enfant-m|Le rond, maintenant !
 copine|Non.
-narrateur|Amir regarde papa.
-papa|On peut proposer.
-maman|On peut accepter plusieurs réponses.
-papa|Oui.
-papa|Non.
-papa|Regarder.
-papa|Plus tard.
-enfant-m|D'accord.
-narrateur|Amir pose un raisin.
-narrateur|Un autre raisin roule sous le bol.
+narrateur|Amir tend le raisin trop vite.
+narrateur|Le raisin glisse sous le bol.
 enfant-m|Il est parti.
-papa|Tu as vu le raisin, Amir ?
+narrateur|L'éclat de grille saute près du bol.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le rond avec Sarah ?
+enfant-m|Oui, papa.
+maman|Tes doigts sont collants ?
+enfant-m|Oui, maman.
+papa|Tu tiens ma manche ?
 enfant-m|Oui.
-narrateur|Amir penche le bol.
-narrateur|Le raisin revient, tout collant.
-maman|Tu proposes encore, tout doux ?
-enfant-m|Tu as vu le gâteau, Sarah ?
-copine|Je regarde.
-papa|Regarder, c'est une réponse.</t>
+narrateur|Amir veut recommencer tout de suite.
+narrateur|Ses doigts foncent vers Sarah.
+enfant-m|Je veux qu'elle pose un raisin !</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>four,cuisine</t>
+          <t>four,vanille,grille</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1426,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir invite Sarah. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir invite &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Côme invite Dounia. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir invite &lt;emphasis&gt;Sarah&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1436,7 +1456,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut proposer. On peut accepter. Que fait-on ?</t>
+          <t>On peut proposer. On peut inviter. Que fait Amir ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1474,7 +1494,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,10 +1502,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1500,34 +1520,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,23 +1560,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=inviter_c_est_proposer_sans_forcer; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1585,17 +1609,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir a su proposer. Il accepte plusieurs réponses. D'accord. Sarah s'assoit près du buffet. Elle regarde le rond. Le rond a trois raisins. Il en manque, hein ? Oui. Tu veux un raisin ? Plus tard. D'accord. Plusieurs réponses sont possibles. Plus tard, au balcon, l'air est frais. Une jardinière sent la terre. Un arrosoir rouge s'appuie au rebord. Amir se souvient. Tu veux l'arrosoir ? Je regarde. On accepte plusieurs réponses. Amir soulève l'arrosoir. Une goutte tombe sur la pierre. C'est bien. Plus tard, tu viens ? Plus tard. D'accord.</t>
+          <t>Amir pousse le raisin vers la main de Sarah. Le raisin colle à son doigt. Non. Sarah retire la main. Le sourire ne revient pas. Amir refuse de foncer. Il pose le raisin près du bol. Personne ne dit la suite. Il écoute le tic de la grille. Il regarde le gâteau, puis Sarah. Sur un fil, l'éclat de grille revient. Tu as vu le gâteau, Sarah ? Je regarde. Sarah s'assoit près du buffet. Elle regarde le rond, sans bouger. D'accord. Amir penche le bol. Le raisin revient, collant. Il pose un raisin sur le gâteau. Le rond a trois raisins. Il en manque, hein ? Oui. Tu veux un raisin ? Plus tard. D'accord. Merci, Amir. Papa a regardé jusqu'au bout. On sort un moment ? Le gâteau vient avec nous. Je porte la grille, à deux mains. Pas trop vite. Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir a su proposer. Il accepte plusieurs réponses. D'accord. Sarah s'assoit près du buffet. Elle regarde le rond. Le rond a trois raisins. Il en manque, hein ? Oui. Tu veux un raisin ? Plus tard. D'accord. Plusieurs réponses sont possibles. Plus tard, au balcon, l'air est frais. Une jardinière sent la terre. Un arrosoir rouge s'appuie au rebord. Amir se souvient. Tu veux l'arrosoir ? Je regarde. On accepte plusieurs réponses. Amir soulève l'arrosoir. Une goutte tombe sur la pierre. C'est bien. Plus tard, tu viens ? Plus tard. D'accord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pousse le raisin vers la main de Sarah. Le raisin colle à son doigt. Non. Sarah retire la main. Le sourire ne revient pas. Amir refuse de foncer. Il pose le raisin près du bol. Personne ne dit la suite. Il écoute le tic de la grille. Il regarde le gâteau, puis Sarah. Sur un fil, l'éclat de grille revient. Tu as vu le gâteau, Sarah ? Je regarde. Sarah s'assoit près du buffet. Elle regarde le rond, sans bouger. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Amir penche le bol. Le raisin revient, collant. Il pose un raisin sur le gâteau. Le rond a trois raisins. Il en manque, hein ? Oui. Tu veux un raisin ? Plus tard. D'accord. Merci, Amir. Papa a regardé jusqu'au bout. On sort un moment ? Le gâteau vient avec nous. Je porte la grille, à deux mains. Pas trop vite. Le ventre d'Amir se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Côme a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Dounia a dit non, puis regarder, puis plus tard. Côme a pu accepter plusieurs réponses. Au jardin aussi. [pause]</t>
+          <t>Amir pousse le raisin vers la main de Sarah. Le raisin colle à son doigt. Non. Sarah retire la main. Le sourire ne revient pas. Amir refuse de foncer. Il pose le raisin près du bol. Personne ne dit la suite. Il écoute le tic de la grille. Il regarde le gâteau, puis Sarah. Sur un fil, l'éclat de grille revient. Tu as vu le gâteau, Sarah ? Je regarde. Sarah s'assoit près du buffet. Elle regarde le rond, sans bouger. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Amir penche le bol. Le raisin revient, collant. Il pose un raisin sur le gâteau. Le rond a trois raisins. Il en manque, hein ? Oui. Tu veux un raisin ? Plus tard. D'accord. Merci, Amir. Papa a regardé jusqu'au bout. On sort un moment ? Le gâteau vient avec nous. Je porte la grille, à deux mains. Pas trop vite. Le ventre d'Amir se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,7 +1666,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1650,10 +1674,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1676,30 +1700,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1708,10 +1732,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1724,41 +1748,48 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_propose_puis_accepte_je_regarde; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir a su proposer.
-narrateur|Il accepte plusieurs réponses.
+          <t>narrateur|Amir pousse le raisin vers la main de Sarah.
+narrateur|Le raisin colle à son doigt.
+copine|Non.
+narrateur|Sarah retire la main.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il pose le raisin près du bol.
+narrateur|Personne ne dit la suite.
+narrateur|Il écoute le tic de la grille.
+narrateur|Il regarde le gâteau, puis Sarah.
+narrateur|Sur un fil, l'éclat de grille revient.
+enfant-m|Tu as vu le gâteau, Sarah ?
+copine|Je regarde.
+narrateur|Sarah s'assoit près du buffet.
+narrateur|Elle regarde le rond, sans bouger.
 enfant-m|D'accord.
-narrateur|Sarah s'assoit près du buffet.
-narrateur|Elle regarde le rond.
+narrateur|Amir penche le bol.
+narrateur|Le raisin revient, collant.
+narrateur|Il pose un raisin sur le gâteau.
 narrateur|Le rond a trois raisins.
 maman|Il en manque, hein ?
 enfant-m|Oui.
 enfant-m|Tu veux un raisin ?
 copine|Plus tard.
 enfant-m|D'accord.
-papa|Plusieurs réponses sont possibles.
-narrateur|Plus tard, au balcon, l'air est frais.
-narrateur|Une jardinière sent la terre.
-narrateur|Un arrosoir rouge s'appuie au rebord.
-narrateur|Amir se souvient.
-enfant-m|Tu veux l'arrosoir ?
-copine|Je regarde.
-maman|On accepte plusieurs réponses.
-narrateur|Amir soulève l'arrosoir.
-narrateur|Une goutte tombe sur la pierre.
-papa|C'est bien.
-enfant-m|Plus tard, tu viens ?
-copine|Plus tard.
-enfant-m|D'accord.</t>
+papa|Merci, Amir.
+narrateur|Papa a regardé jusqu'au bout.
+maman|On sort un moment ?
+enfant-m|Le gâteau vient avec nous.
+papa|Je porte la grille, à deux mains.
+enfant-m|Pas trop vite.
+narrateur|Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>balcon</t>
+          <t>raisins,grille</t>
         </is>
       </c>
     </row>
@@ -1785,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent près du gâteau. La vanille est plus douce, maintenant. Sarah hoche la tête. Elle pose un raisin. Le raisin colle un peu. Puis elle s'arrête. Amir accepte. Tu as su proposer. Tu as su accepter. Bravo, Amir. Amir pose le dernier raisin. Le rond est fini. Il brille un peu, au milieu. Il est rond, papa. Oui. Tout autour. On range le bol ? Oui. Sarah range un raisin tombé. Tu as fini le rond, Amir ? Oui, papa. La vanille sent encore, tout doux.</t>
+          <t>Au balcon, l'air est frais. La vanille suit, plus légère. Papa pose la grille sur la table. Une jardinière sent la terre. Le rond, Sarah ! Amir veut le dernier raisin, d'un coup. Il pousse le bol trop vite. Un raisin file vers le bord. Ça roule ! Le gâteau glisse d'un fil. Oh. Amir veut le rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la grille, il écoute le balcon. Un oiseau passe, loin. Tu poses celui-là ? Sarah ne dit rien. Elle garde les mains sur ses genoux. D'accord. Amir attend. Plus tard. Oui. Le gâteau se cale, sans glisser. Sarah avance un doigt. Elle pose un raisin, puis s'arrête. D'accord. Amir pose le dernier raisin. Il est rond, papa. Tu le vois, autour ? Oui. Tes pieds sont sous la table ? Oui, maman. Le tic est là. Le rond, lui, reste.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent près du gâteau. La vanille est plus douce, maintenant. Sarah hoche la tête. Elle pose un raisin. Le raisin colle un peu. Puis elle s'arrête. Amir accepte. Tu as su proposer. Tu as su accepter. Bravo, Amir. Amir pose le dernier raisin. Le rond est fini. Il brille un peu, au milieu. Il est rond, papa. Oui. Tout autour. On range le bol ? Oui. Sarah range un raisin tombé. Tu as fini le rond, Amir ? Oui, papa. La vanille sent encore, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au balcon, l'air est frais. La vanille suit, plus légère. Papa pose la grille sur la table. Une jardinière sent la terre. Le rond, Sarah ! Amir veut le dernier &lt;emphasis level="moderate"&gt;raisin&lt;/emphasis&gt;, d'un coup. Il pousse le bol trop vite. Un raisin file vers le bord. Ça roule ! Le gâteau glisse d'un fil. Oh. Amir veut le rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la grille, il écoute le balcon. Un oiseau passe, loin. Tu poses celui-là ? Sarah ne dit rien. Elle garde les mains sur ses genoux. D'accord. Amir attend. Plus tard. Oui. Le gâteau se cale, sans glisser. Sarah avance un doigt. Elle pose un raisin, puis s'arrête. D'accord. Amir pose le dernier raisin. Il est rond, papa. Tu le vois, autour ? Oui. Tes pieds sont sous la table ? Oui, maman. Le tic est là. Le rond, lui, reste.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman dit : on range. Côme pose le cerceau. Dounia range un crayon. Ils se disent merci. [pause]</t>
+          <t>Au balcon, l'air est frais. La vanille suit, plus légère. Papa pose la grille sur la table. Une jardinière sent la terre. Le rond, Sarah ! Amir veut le dernier &lt;emphasis&gt;raisin&lt;/emphasis&gt;, d'un coup. Il pousse le bol trop vite. Un raisin file vers le bord. Ça roule ! Le gâteau glisse d'un fil. Oh. Amir veut le rattraper, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde la grille, il écoute le balcon. Un oiseau passe, loin. Tu poses celui-là ? Sarah ne dit rien. Elle garde les mains sur ses genoux. D'accord. Amir attend. Plus tard. Oui. Le gâteau se cale, sans glisser. Sarah avance un doigt. Elle pose un raisin, puis s'arrête. D'accord. Amir pose le dernier raisin. Il est rond, papa. Tu le vois, autour ? Oui. Tes pieds sont sous la table ? Oui, maman. Le tic est là. Le rond, lui, reste. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1842,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1850,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1874,28 +1905,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>raisin</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,10 +1939,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1918,36 +1953,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_rattraper_trop_vite; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils rentrent près du gâteau.
-narrateur|La vanille est plus douce, maintenant.
-narrateur|Sarah hoche la tête.
-narrateur|Elle pose un raisin.
-narrateur|Le raisin colle un peu.
-narrateur|Puis elle s'arrête.
-narrateur|Amir accepte.
-maman|Tu as su proposer.
-papa|Tu as su accepter.
-maman|Bravo, Amir.
+          <t>narrateur|Au balcon, l'air est frais.
+narrateur|La vanille suit, plus légère.
+narrateur|Papa pose la grille sur la table.
+narrateur|Une jardinière sent la terre.
+enfant-m|Le rond, Sarah !
+narrateur|Amir veut le dernier raisin, d'un coup.
+narrateur|Il pousse le bol trop vite.
+narrateur|Un raisin file vers le bord.
+enfant-m|Ça roule !
+narrateur|Le gâteau glisse d'un fil.
+enfant-m|Oh.
+narrateur|Amir veut le rattraper, d'un coup.
+narrateur|Amir refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Il regarde la grille, il écoute le balcon.
+narrateur|Un oiseau passe, loin.
+enfant-m|Tu poses celui-là ?
+narrateur|Sarah ne dit rien.
+narrateur|Elle garde les mains sur ses genoux.
+enfant-m|D'accord.
+narrateur|Amir attend.
+copine|Plus tard.
+enfant-m|Oui.
+narrateur|Le gâteau se cale, sans glisser.
+narrateur|Sarah avance un doigt.
+narrateur|Elle pose un raisin, puis s'arrête.
+enfant-m|D'accord.
 narrateur|Amir pose le dernier raisin.
-narrateur|Le rond est fini.
-narrateur|Il brille un peu, au milieu.
 enfant-m|Il est rond, papa.
-papa|Oui.
-papa|Tout autour.
-maman|On range le bol ?
+papa|Tu le vois, autour ?
 enfant-m|Oui.
-narrateur|Sarah range un raisin tombé.
-papa|Tu as fini le rond, Amir ?
-enfant-m|Oui, papa.
-narrateur|La vanille sent encore, tout doux.</t>
+maman|Tes pieds sont sous la table ?
+enfant-m|Oui, maman.
+papa|Le tic est là.
+enfant-m|Le rond, lui, reste.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>cuisine</t>
+          <t>balcon</t>
         </is>
       </c>
     </row>
@@ -1974,17 +2028,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le gâteau a son rond de raisins. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. L'arrosoir rouge s'appuie encore au rebord.</t>
+          <t>Ils restent près de la table. Le gâteau a son rond de raisins. L'éclat est là, papa. Tu le vois sur le fil ? Oui, papa. On est bien, ici. La vanille reste, plus légère. Il est rond, mon gâteau. Il est rond, Amir. Oui, maman. Amir pose la joue près de la grille. La grille est tiède, un peu. C'est tiède. Tu le sens sur tes joues ? Oui, elle est tiède. Un raisin porte une trace de doigt. Dehors, le balcon s'endort. L'éclat de grille tient sur le fil.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le gâteau a son rond de raisins. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. L'arrosoir rouge s'appuie encore au rebord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Le gâteau a son rond de raisins. L'éclat est là, papa. Tu le vois sur le fil ? Oui, papa. On est bien, ici. La vanille reste, plus légère. Il est rond, mon gâteau. Il est rond, Amir. Oui, maman. Amir pose la joue près de la grille. La grille est tiède, un peu. C'est tiède. Tu le sens sur tes joues ? Oui, elle est tiède. Un raisin porte une trace de doigt. Dehors, le balcon s'endort. L'&lt;emphasis level="moderate"&gt;éclat de grille&lt;/emphasis&gt; tient sur le fil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Le gâteau a son rond de raisins. L'éclat est là, papa. Tu le vois sur le fil ? Oui, papa. On est bien, ici. La vanille reste, plus légère. Il est rond, mon gâteau. Il est rond, Amir. Oui, maman. Amir pose la joue près de la grille. La grille est tiède, un peu. C'est tiède. Tu le sens sur tes joues ? Oui, elle est tiède. Un raisin porte une trace de doigt. Dehors, le balcon s'endort. L'&lt;emphasis&gt;éclat de grille&lt;/emphasis&gt; tient sur le fil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2031,18 +2085,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2051,12 +2105,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2065,17 +2119,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de grille</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2084,11 +2142,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2097,29 +2155,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fil; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le gâteau a son rond de raisins.
-enfant-m|J'ai proposé.
-enfant-m|J'ai accepté.
-maman|Plusieurs réponses sont possibles.
-papa|Oui.
-narrateur|L'arrosoir rouge s'appuie encore au rebord.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Le gâteau a son rond de raisins.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur le fil ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|La vanille reste, plus légère.
+enfant-m|Il est rond, mon gâteau.
+maman|Il est rond, Amir.
+enfant-m|Oui, maman.
+narrateur|Amir pose la joue près de la grille.
+narrateur|La grille est tiède, un peu.
+enfant-m|C'est tiède.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, elle est tiède.
+narrateur|Un raisin porte une trace de doigt.
+narrateur|Dehors, le balcon s'endort.
+narrateur|L'éclat de grille tient sur le fil.</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2292,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>